<commit_message>
Add 2026 tab to GP_by_Buyer_Final.xlsx, rename Cumulative to 2024-25 Cumulative
</commit_message>
<xml_diff>
--- a/Trading Analysis/LAM Billings Review/CM Billings/Final/GP_by_Buyer_Final.xlsx
+++ b/Trading Analysis/LAM Billings Review/CM Billings/Final/GP_by_Buyer_Final.xlsx
@@ -5,7 +5,8 @@
   <sheets>
     <sheet name="2024" sheetId="1" r:id="rId1"/>
     <sheet name="2025" sheetId="2" r:id="rId2"/>
-    <sheet name="Cumulative" sheetId="3" r:id="rId3"/>
+    <sheet name="2026" sheetId="3" r:id="rId3"/>
+    <sheet name="2024-25 Cumulative" sheetId="4" r:id="rId4"/>
   </sheets>
 </workbook>
 </file>
@@ -743,6 +744,155 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:E9"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>Buyer</v>
+      </c>
+      <c r="B1" t="str">
+        <v>JABIL GP</v>
+      </c>
+      <c r="C1" t="str">
+        <v>Naprotek GP</v>
+      </c>
+      <c r="D1" t="str">
+        <v>VM Services GP</v>
+      </c>
+      <c r="E1" t="str">
+        <v>Total Lines</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>Tracy Xie</v>
+      </c>
+      <c r="C2">
+        <v>8.51</v>
+      </c>
+      <c r="D2">
+        <v>11367.16</v>
+      </c>
+      <c r="E2">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>Jake Harris</v>
+      </c>
+      <c r="B3">
+        <v>-307.29</v>
+      </c>
+      <c r="C3">
+        <v>546.77</v>
+      </c>
+      <c r="D3">
+        <v>4196.31</v>
+      </c>
+      <c r="E3">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>DM</v>
+      </c>
+      <c r="C4">
+        <v>3.46</v>
+      </c>
+      <c r="D4">
+        <v>640.07</v>
+      </c>
+      <c r="E4">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>Stephanie Hill</v>
+      </c>
+      <c r="B5">
+        <v>-164.66</v>
+      </c>
+      <c r="C5">
+        <v>93.2</v>
+      </c>
+      <c r="D5">
+        <v>466.35</v>
+      </c>
+      <c r="E5">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>Edgar Santana</v>
+      </c>
+      <c r="C6">
+        <v>9.22</v>
+      </c>
+      <c r="D6">
+        <v>216.01</v>
+      </c>
+      <c r="E6">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>SZ</v>
+      </c>
+      <c r="D7">
+        <v>8.39</v>
+      </c>
+      <c r="E7">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>TOTAL GP</v>
+      </c>
+      <c r="B8">
+        <v>-471.94</v>
+      </c>
+      <c r="C8">
+        <v>661.17</v>
+      </c>
+      <c r="D8">
+        <v>16894.29</v>
+      </c>
+      <c r="E8">
+        <v>291</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>MARGIN</v>
+      </c>
+      <c r="B9">
+        <v>-0.24600000000000002</v>
+      </c>
+      <c r="C9">
+        <v>0.361</v>
+      </c>
+      <c r="D9">
+        <v>0.423</v>
+      </c>
+      <c r="E9">
+        <v>0.391</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:E9"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:G6"/>
   <sheetData>
     <row r="1">

</xml_diff>

<commit_message>
Merge Daniel and DM (Danyel) into Edgar Santana across all GP files
</commit_message>
<xml_diff>
--- a/Trading Analysis/LAM Billings Review/CM Billings/Final/GP_by_Buyer_Final.xlsx
+++ b/Trading Analysis/LAM Billings Review/CM Billings/Final/GP_by_Buyer_Final.xlsx
@@ -400,7 +400,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G7"/>
+  <dimension ref="A1:G6"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -453,19 +453,19 @@
         <v>Edgar Santana</v>
       </c>
       <c r="B3">
-        <v>23</v>
+        <v>36</v>
       </c>
       <c r="C3">
-        <v>2769</v>
-      </c>
-      <c r="D3" t="str">
-        <v>24.6%</v>
+        <v>2894.87</v>
+      </c>
+      <c r="D3">
+        <v>63.1</v>
       </c>
       <c r="E3">
-        <v>2291.62</v>
+        <v>2308.64</v>
       </c>
       <c r="F3">
-        <v>400.18</v>
+        <v>509.03</v>
       </c>
       <c r="G3">
         <v>77.2</v>
@@ -496,22 +496,22 @@
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>Daniel</v>
+        <v>Tracy Xie</v>
       </c>
       <c r="B5">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="C5">
-        <v>125.87</v>
+        <v>97.98</v>
       </c>
       <c r="D5" t="str">
-        <v>38.5%</v>
-      </c>
-      <c r="E5">
-        <v>17.02</v>
+        <v>8.5%</v>
+      </c>
+      <c r="E5" t="str">
+        <v/>
       </c>
       <c r="F5">
-        <v>108.85</v>
+        <v>97.98</v>
       </c>
       <c r="G5" t="str">
         <v/>
@@ -519,60 +519,37 @@
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>Tracy Xie</v>
+        <v>TOTAL</v>
       </c>
       <c r="B6">
-        <v>6</v>
+        <v>130</v>
       </c>
       <c r="C6">
-        <v>97.98</v>
+        <v>8151.03</v>
       </c>
       <c r="D6" t="str">
-        <v>8.5%</v>
-      </c>
-      <c r="E6" t="str">
-        <v/>
+        <v>33.3%</v>
+      </c>
+      <c r="E6">
+        <v>2758.02</v>
       </c>
       <c r="F6">
-        <v>97.98</v>
-      </c>
-      <c r="G6" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="str">
-        <v>TOTAL</v>
-      </c>
-      <c r="B7">
-        <v>130</v>
-      </c>
-      <c r="C7">
-        <v>8151.03</v>
-      </c>
-      <c r="D7" t="str">
-        <v>33.3%</v>
-      </c>
-      <c r="E7">
-        <v>2758.02</v>
-      </c>
-      <c r="F7">
         <v>4760.47</v>
       </c>
-      <c r="G7">
+      <c r="G6">
         <v>632.54</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G7"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G6"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G7"/>
+  <dimension ref="A1:G6"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -671,109 +648,86 @@
         <v>Edgar Santana</v>
       </c>
       <c r="B5">
-        <v>52</v>
+        <v>80</v>
       </c>
       <c r="C5">
-        <v>872.94</v>
-      </c>
-      <c r="D5" t="str">
-        <v>28.8%</v>
+        <v>1259.17</v>
+      </c>
+      <c r="D5">
+        <v>43.3</v>
       </c>
       <c r="E5">
-        <v>170.09</v>
+        <v>356.94</v>
       </c>
       <c r="F5">
-        <v>493.42</v>
+        <v>629.21</v>
       </c>
       <c r="G5">
-        <v>209.43</v>
+        <v>273.03000000000003</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>Daniel</v>
+        <v>TOTAL</v>
       </c>
       <c r="B6">
-        <v>28</v>
+        <v>469</v>
       </c>
       <c r="C6">
-        <v>386.23</v>
+        <v>16830.95</v>
       </c>
       <c r="D6" t="str">
-        <v>14.5%</v>
+        <v>39.9%</v>
       </c>
       <c r="E6">
-        <v>186.85</v>
+        <v>2115.52</v>
       </c>
       <c r="F6">
-        <v>135.79</v>
+        <v>14019.76</v>
       </c>
       <c r="G6">
-        <v>63.6</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="str">
-        <v>TOTAL</v>
-      </c>
-      <c r="B7">
-        <v>469</v>
-      </c>
-      <c r="C7">
-        <v>16830.95</v>
-      </c>
-      <c r="D7" t="str">
-        <v>39.9%</v>
-      </c>
-      <c r="E7">
-        <v>2115.52</v>
-      </c>
-      <c r="F7">
-        <v>14019.76</v>
-      </c>
-      <c r="G7">
         <v>695.67</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G7"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G6"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E9"/>
+  <dimension ref="A1:E8"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
         <v>Buyer</v>
       </c>
       <c r="B1" t="str">
+        <v>Naprotek GP</v>
+      </c>
+      <c r="C1" t="str">
+        <v>VM Services GP</v>
+      </c>
+      <c r="D1" t="str">
+        <v>Total Lines</v>
+      </c>
+      <c r="E1" t="str">
         <v>JABIL GP</v>
-      </c>
-      <c r="C1" t="str">
-        <v>Naprotek GP</v>
-      </c>
-      <c r="D1" t="str">
-        <v>VM Services GP</v>
-      </c>
-      <c r="E1" t="str">
-        <v>Total Lines</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
         <v>Tracy Xie</v>
       </c>
+      <c r="B2">
+        <v>8.51</v>
+      </c>
       <c r="C2">
-        <v>8.51</v>
+        <v>11367.16</v>
       </c>
       <c r="D2">
-        <v>11367.16</v>
-      </c>
-      <c r="E2">
         <v>33</v>
       </c>
     </row>
@@ -782,111 +736,97 @@
         <v>Jake Harris</v>
       </c>
       <c r="B3">
+        <v>546.77</v>
+      </c>
+      <c r="C3">
+        <v>4196.31</v>
+      </c>
+      <c r="D3">
+        <v>118</v>
+      </c>
+      <c r="E3">
         <v>-307.29</v>
-      </c>
-      <c r="C3">
-        <v>546.77</v>
-      </c>
-      <c r="D3">
-        <v>4196.31</v>
-      </c>
-      <c r="E3">
-        <v>118</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>DM</v>
+        <v>Stephanie Hill</v>
+      </c>
+      <c r="B4">
+        <v>93.2</v>
       </c>
       <c r="C4">
-        <v>3.46</v>
+        <v>466.35</v>
       </c>
       <c r="D4">
-        <v>640.07</v>
+        <v>94</v>
       </c>
       <c r="E4">
-        <v>19</v>
+        <v>-164.66</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>Stephanie Hill</v>
+        <v>Edgar Santana</v>
       </c>
       <c r="B5">
-        <v>-164.66</v>
+        <v>12.68</v>
       </c>
       <c r="C5">
-        <v>93.2</v>
+        <v>856.08</v>
       </c>
       <c r="D5">
-        <v>466.35</v>
-      </c>
-      <c r="E5">
-        <v>94</v>
+        <v>44</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>Edgar Santana</v>
+        <v>SZ</v>
       </c>
       <c r="C6">
-        <v>9.22</v>
+        <v>8.39</v>
       </c>
       <c r="D6">
-        <v>216.01</v>
-      </c>
-      <c r="E6">
-        <v>25</v>
+        <v>2</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>SZ</v>
+        <v>TOTAL GP</v>
+      </c>
+      <c r="B7">
+        <v>661.17</v>
+      </c>
+      <c r="C7">
+        <v>16894.29</v>
       </c>
       <c r="D7">
-        <v>8.39</v>
+        <v>291</v>
       </c>
       <c r="E7">
-        <v>2</v>
+        <v>-471.94</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>TOTAL GP</v>
+        <v>MARGIN</v>
       </c>
       <c r="B8">
-        <v>-471.94</v>
+        <v>0.361</v>
       </c>
       <c r="C8">
-        <v>661.17</v>
+        <v>0.423</v>
       </c>
       <c r="D8">
-        <v>16894.29</v>
+        <v>0.391</v>
       </c>
       <c r="E8">
-        <v>291</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="str">
-        <v>MARGIN</v>
-      </c>
-      <c r="B9">
         <v>-0.24600000000000002</v>
-      </c>
-      <c r="C9">
-        <v>0.361</v>
-      </c>
-      <c r="D9">
-        <v>0.423</v>
-      </c>
-      <c r="E9">
-        <v>0.391</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E9"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E8"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add Total GP and Total Margin columns to 2026 GP by Buyer data
</commit_message>
<xml_diff>
--- a/Trading Analysis/LAM Billings Review/CM Billings/Final/GP_by_Buyer_Final.xlsx
+++ b/Trading Analysis/LAM Billings Review/CM Billings/Final/GP_by_Buyer_Final.xlsx
@@ -698,22 +698,28 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:G7"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
         <v>Buyer</v>
       </c>
       <c r="B1" t="str">
+        <v>Total Lines</v>
+      </c>
+      <c r="C1" t="str">
+        <v>Total GP</v>
+      </c>
+      <c r="D1" t="str">
+        <v>Total Margin</v>
+      </c>
+      <c r="E1" t="str">
+        <v>VM Services GP</v>
+      </c>
+      <c r="F1" t="str">
         <v>Naprotek GP</v>
       </c>
-      <c r="C1" t="str">
-        <v>VM Services GP</v>
-      </c>
-      <c r="D1" t="str">
-        <v>Total Lines</v>
-      </c>
-      <c r="E1" t="str">
+      <c r="G1" t="str">
         <v>JABIL GP</v>
       </c>
     </row>
@@ -722,13 +728,19 @@
         <v>Tracy Xie</v>
       </c>
       <c r="B2">
+        <v>33</v>
+      </c>
+      <c r="C2">
+        <v>11375.67</v>
+      </c>
+      <c r="D2">
+        <v>0.423</v>
+      </c>
+      <c r="E2">
+        <v>11367.16</v>
+      </c>
+      <c r="F2">
         <v>8.51</v>
-      </c>
-      <c r="C2">
-        <v>11367.16</v>
-      </c>
-      <c r="D2">
-        <v>33</v>
       </c>
     </row>
     <row r="3">
@@ -736,15 +748,21 @@
         <v>Jake Harris</v>
       </c>
       <c r="B3">
+        <v>118</v>
+      </c>
+      <c r="C3">
+        <v>4435.79</v>
+      </c>
+      <c r="D3">
+        <v>0.326</v>
+      </c>
+      <c r="E3">
+        <v>4196.31</v>
+      </c>
+      <c r="F3">
         <v>546.77</v>
       </c>
-      <c r="C3">
-        <v>4196.31</v>
-      </c>
-      <c r="D3">
-        <v>118</v>
-      </c>
-      <c r="E3">
+      <c r="G3">
         <v>-307.29</v>
       </c>
     </row>
@@ -753,15 +771,21 @@
         <v>Stephanie Hill</v>
       </c>
       <c r="B4">
+        <v>94</v>
+      </c>
+      <c r="C4">
+        <v>394.89</v>
+      </c>
+      <c r="D4">
+        <v>0.08199999999999999</v>
+      </c>
+      <c r="E4">
+        <v>466.35</v>
+      </c>
+      <c r="F4">
         <v>93.2</v>
       </c>
-      <c r="C4">
-        <v>466.35</v>
-      </c>
-      <c r="D4">
-        <v>94</v>
-      </c>
-      <c r="E4">
+      <c r="G4">
         <v>-164.66</v>
       </c>
     </row>
@@ -770,63 +794,64 @@
         <v>Edgar Santana</v>
       </c>
       <c r="B5">
+        <v>44</v>
+      </c>
+      <c r="C5">
+        <v>868.76</v>
+      </c>
+      <c r="D5">
+        <v>0.381</v>
+      </c>
+      <c r="E5">
+        <v>856.08</v>
+      </c>
+      <c r="F5">
         <v>12.68</v>
-      </c>
-      <c r="C5">
-        <v>856.08</v>
-      </c>
-      <c r="D5">
-        <v>44</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>SZ</v>
+        <v>Serena Zhang</v>
+      </c>
+      <c r="B6">
+        <v>2</v>
       </c>
       <c r="C6">
         <v>8.39</v>
       </c>
       <c r="D6">
-        <v>2</v>
+        <v>0.18</v>
+      </c>
+      <c r="E6">
+        <v>8.39</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>TOTAL GP</v>
+        <v>TOTAL</v>
       </c>
       <c r="B7">
+        <v>291</v>
+      </c>
+      <c r="C7">
+        <v>17083.5</v>
+      </c>
+      <c r="D7">
+        <v>0.391</v>
+      </c>
+      <c r="E7">
+        <v>16894.29</v>
+      </c>
+      <c r="F7">
         <v>661.17</v>
       </c>
-      <c r="C7">
-        <v>16894.29</v>
-      </c>
-      <c r="D7">
-        <v>291</v>
-      </c>
-      <c r="E7">
+      <c r="G7">
         <v>-471.94</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="str">
-        <v>MARGIN</v>
-      </c>
-      <c r="B8">
-        <v>0.361</v>
-      </c>
-      <c r="C8">
-        <v>0.423</v>
-      </c>
-      <c r="D8">
-        <v>0.391</v>
-      </c>
-      <c r="E8">
-        <v>-0.24600000000000002</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E8"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G7"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>